<commit_message>
Atualização semanal — Round 12
</commit_message>
<xml_diff>
--- a/Perth_SC_GPS_Weekly_Update_v3.xlsx
+++ b/Perth_SC_GPS_Weekly_Update_v3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thali/Desktop/Perth_Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37402A4B-EE46-B64C-8A12-3CA00D92EECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41535D13-C404-E144-8973-EAFDA1B8524E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GPS Data" sheetId="1" r:id="rId1"/>
@@ -547,20 +547,20 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1967,52 +1967,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
     </row>
     <row r="5" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
       <c r="J5" s="4" t="s">
         <v>4</v>
       </c>
@@ -2616,14 +2616,14 @@
       </c>
     </row>
     <row r="29" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="28"/>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="27"/>
+      <c r="A29" s="30"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="28"/>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
     </row>
@@ -2800,14 +2800,14 @@
       <c r="H45" s="21"/>
     </row>
     <row r="52" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="28"/>
-      <c r="B52" s="27"/>
-      <c r="C52" s="27"/>
-      <c r="D52" s="27"/>
-      <c r="E52" s="27"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="27"/>
-      <c r="H52" s="27"/>
+      <c r="A52" s="30"/>
+      <c r="B52" s="28"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="28"/>
+      <c r="E52" s="28"/>
+      <c r="F52" s="28"/>
+      <c r="G52" s="28"/>
+      <c r="H52" s="28"/>
       <c r="J52" s="4"/>
       <c r="K52" s="4"/>
     </row>
@@ -2975,12 +2975,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A52:H52"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A52:H52"/>
   </mergeCells>
   <conditionalFormatting sqref="G7:G22">
     <cfRule type="dataBar" priority="1">
@@ -3025,7 +3025,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="26" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>